<commit_message>
Cambio descripción en excel.
</commit_message>
<xml_diff>
--- a/docs/ejercicio2.xlsx
+++ b/docs/ejercicio2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Z PROYECTOS\UVG\Semestre 2\ejercicio2\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CCF2040-9FD1-4BF9-807F-A13981F92139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A417B04B-5EDC-462E-A221-3B5DA108FE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="16090" activeTab="1" xr2:uid="{54BB8998-16D7-4C75-86AC-D8865F1E09BB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{54BB8998-16D7-4C75-86AC-D8865F1E09BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Clases MVC" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="140">
   <si>
     <t>Clase</t>
   </si>
@@ -130,9 +130,6 @@
   </si>
   <si>
     <t>vista</t>
-  </si>
-  <si>
-    <t>Diagrama UML</t>
   </si>
   <si>
     <t>Atleta</t>
@@ -665,6 +662,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -673,15 +679,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1040,46 +1037,46 @@
         <v>26</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="2:6">
@@ -1093,22 +1090,20 @@
         <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="F7" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="D8" s="3"/>
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="1"/>
@@ -1134,14 +1129,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7">
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="17"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="2:7">
       <c r="B2" s="4" t="s">
@@ -1164,21 +1159,21 @@
       </c>
     </row>
     <row r="3" spans="2:7">
-      <c r="B3" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="14"/>
+      <c r="B3" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="17"/>
     </row>
     <row r="4" spans="2:7">
       <c r="B4" s="2">
         <v>1</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>12</v>
@@ -1190,7 +1185,7 @@
         <v>14</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="2:7">
@@ -1198,7 +1193,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>15</v>
@@ -1210,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="2:7">
@@ -1218,7 +1213,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>15</v>
@@ -1230,7 +1225,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="2:7">
@@ -1238,7 +1233,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>15</v>
@@ -1250,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="19.5" customHeight="1">
@@ -1258,70 +1253,70 @@
         <v>5</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="2:7">
-      <c r="B9" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="14"/>
+      <c r="B9" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17"/>
     </row>
     <row r="10" spans="2:7">
       <c r="B10" s="2">
         <v>1</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>81</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>83</v>
-      </c>
     </row>
     <row r="11" spans="2:7">
-      <c r="B11" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="14"/>
+      <c r="B11" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17"/>
     </row>
     <row r="12" spans="2:7">
       <c r="B12" s="2">
         <v>1</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>13</v>
@@ -1330,7 +1325,7 @@
         <v>22</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="15" customHeight="1">
@@ -1341,16 +1336,16 @@
         <v>29</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F13" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="15" customHeight="1">
@@ -1358,7 +1353,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>15</v>
@@ -1370,7 +1365,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="2:7">
@@ -1383,7 +1378,7 @@
     </row>
     <row r="16" spans="2:7">
       <c r="B16" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="18"/>
@@ -1392,14 +1387,14 @@
       <c r="G16" s="18"/>
     </row>
     <row r="18" spans="2:7">
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="17"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="14"/>
     </row>
     <row r="19" spans="2:7">
       <c r="B19" s="4" t="s">
@@ -1422,31 +1417,31 @@
       </c>
     </row>
     <row r="20" spans="2:7">
-      <c r="B20" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="14"/>
+      <c r="B20" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17"/>
     </row>
     <row r="21" spans="2:7" ht="14" customHeight="1">
       <c r="B21" s="2">
         <v>1</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="2:7">
@@ -1454,19 +1449,19 @@
         <v>2</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1">
@@ -1474,19 +1469,19 @@
         <v>3</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>27</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="15" customHeight="1">
@@ -1494,19 +1489,19 @@
         <v>4</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>16</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="2:7">
@@ -1514,7 +1509,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>27</v>
@@ -1524,7 +1519,7 @@
         <v>25</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="2:7">
@@ -1532,7 +1527,7 @@
         <v>6</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>27</v>
@@ -1542,7 +1537,7 @@
         <v>25</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="2:7">
@@ -1550,7 +1545,7 @@
         <v>7</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>27</v>
@@ -1560,7 +1555,7 @@
         <v>25</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="2:7">
@@ -1568,7 +1563,7 @@
         <v>8</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>15</v>
@@ -1578,7 +1573,7 @@
         <v>25</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="2:7">
@@ -1586,7 +1581,7 @@
         <v>9</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>15</v>
@@ -1596,7 +1591,7 @@
         <v>25</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="2:7">
@@ -1604,7 +1599,7 @@
         <v>10</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>12</v>
@@ -1614,7 +1609,7 @@
         <v>25</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="2:7">
@@ -1622,7 +1617,7 @@
         <v>11</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>15</v>
@@ -1632,7 +1627,7 @@
         <v>25</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="2:7">
@@ -1640,7 +1635,7 @@
         <v>12</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>15</v>
@@ -1650,7 +1645,7 @@
         <v>25</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="2:7">
@@ -1658,49 +1653,49 @@
         <v>13</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>16</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="2:7">
-      <c r="B34" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="14"/>
+      <c r="B34" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="17"/>
     </row>
     <row r="35" spans="2:7">
       <c r="B35" s="1">
         <v>1</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="2:7">
@@ -1708,19 +1703,19 @@
         <v>2</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="2:7">
@@ -1728,19 +1723,19 @@
         <v>3</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="2:7">
@@ -1748,19 +1743,19 @@
         <v>4</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>12</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="2:7">
@@ -1768,19 +1763,19 @@
         <v>5</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D39" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="2:7">
@@ -1788,19 +1783,19 @@
         <v>6</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="2:7">
@@ -1808,19 +1803,19 @@
         <v>7</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>27</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" spans="2:7">
@@ -1828,19 +1823,19 @@
         <v>8</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="2:7">
@@ -1848,49 +1843,49 @@
         <v>9</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D43" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E43" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G43" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F43" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>101</v>
-      </c>
     </row>
     <row r="44" spans="2:7">
-      <c r="B44" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="14"/>
+      <c r="B44" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="16"/>
+      <c r="G44" s="17"/>
     </row>
     <row r="45" spans="2:7">
       <c r="B45" s="1">
         <v>1</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E45" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G45" s="8" t="s">
         <v>106</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="46" spans="2:7">
@@ -1898,19 +1893,19 @@
         <v>2</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D46" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="47" spans="2:7">
@@ -1918,19 +1913,19 @@
         <v>3</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="2:7">
@@ -1938,19 +1933,19 @@
         <v>4</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49" spans="2:7">
@@ -1958,19 +1953,19 @@
         <v>5</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="2:7">
@@ -1978,19 +1973,19 @@
         <v>6</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D50" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="51" spans="2:7">
@@ -1998,19 +1993,19 @@
         <v>7</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D51" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="52" spans="2:7">
@@ -2018,19 +2013,19 @@
         <v>8</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" spans="2:7">
@@ -2038,19 +2033,19 @@
         <v>9</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="54" spans="2:7">
@@ -2058,63 +2053,63 @@
         <v>10</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D54" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="2:7">
-      <c r="B55" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="14"/>
+      <c r="B55" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="17"/>
     </row>
     <row r="56" spans="2:7">
       <c r="B56" s="1">
         <v>1</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D56" s="9" t="s">
         <v>28</v>
       </c>
       <c r="E56" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F56" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="F56" s="9" t="s">
+      <c r="G56" s="8" t="s">
         <v>128</v>
-      </c>
-      <c r="G56" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B44:G44"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B55:G55"/>
+    <mergeCell ref="B34:G34"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B44:G44"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B55:G55"/>
-    <mergeCell ref="B34:G34"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>